<commit_message>
fix: balance reasoning question answer keys, update excel test, and enhance review screen grid
</commit_message>
<xml_diff>
--- a/public/downloads/Class_7_Reasoning_Visual_Mock_Test.xlsx
+++ b/public/downloads/Class_7_Reasoning_Visual_Mock_Test.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
   <si>
     <t>Subject</t>
   </si>
@@ -58,28 +58,28 @@
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20200%20200%22%20width%3D%22200%22%20height%3D%22200%22%3E%20%3Crect%20width%3D%22200%22%20height%3D%22200%22%20fill%3D%22%23f8fafc%22%20stroke%3D%22%23334155%22%20stroke-width%3D%223%22%20rx%3D%2210%22%2F%3E%20%3Cline%20x1%3D%22100%22%20y1%3D%220%22%20x2%3D%22100%22%20y2%3D%22200%22%20stroke%3D%22%2364748b%22%20stroke-width%3D%222%22%20stroke-dasharray%3D%224%2C4%22%2F%3E%20%3Cline%20x1%3D%220%22%20y1%3D%22100%22%20x2%3D%22200%22%20y2%3D%22100%22%20stroke%3D%22%2364748b%22%20stroke-width%3D%222%22%20stroke-dasharray%3D%224%2C4%22%2F%3E%20%3C!--%20Top%20Left%3A%20Top-left%20quarter%20shaded%20--%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2230%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpath%20d%3D%22M%2050%2050%20L%2050%2020%20A%2030%2030%200%200%200%2020%2050%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C!--%20Top%20Right%3A%20Top-right%20quarter%20shaded%20--%3E%20%3Ccircle%20cx%3D%22150%22%20cy%3D%2250%22%20r%3D%2230%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpath%20d%3D%22M%20150%2050%20L%20180%2050%20A%2030%2030%200%200%200%20150%2020%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C!--%20Bottom%20Left%3A%20Bottom-left%20quarter%20shaded%20--%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%22150%22%20r%3D%2230%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpath%20d%3D%22M%2050%20150%20L%2020%20150%20A%2030%2030%200%200%200%2050%20180%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C!--%20Bottom%20Right%3A%20Question%20Mark%20--%3E%20%3Crect%20x%3D%22105%22%20y%3D%22105%22%20width%3D%2290%22%20height%3D%2290%22%20fill%3D%22%23fef3c7%22%20stroke%3D%22%23f59e0b%22%20stroke-width%3D%222%22%20rx%3D%226%22%2F%3E%20%3Ctext%20x%3D%22150%22%20y%3D%22162%22%20font-size%3D%2244%22%20font-weight%3D%22900%22%20fill%3D%22%23dc2626%22%20text-anchor%3D%22middle%22%20font-family%3D%22sans-serif%22%3E%3F%3C%2Ftext%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2234%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%2F%3E%20%3Cpath%20d%3D%22M%2050%2050%20L%2050%2016%20A%2034%2034%200%200%200%2016%2050%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2234%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%2F%3E%20%3Cpath%20d%3D%22M%2050%2050%20L%2050%2084%20A%2034%2034%200%200%200%2084%2050%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2234%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%2F%3E%20%3Cpath%20d%3D%22M%2050%2050%20L%2050%2016%20A%2034%2034%200%200%200%2016%2050%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2234%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%2F%3E%20%3Cpath%20d%3D%22M%2050%2050%20L%2084%2050%20A%2034%2034%200%200%200%2050%2016%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2234%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%2F%3E%20%3Cpath%20d%3D%22M%2016%2050%20A%2034%2034%200%200%201%2084%2050%20Z%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Option A is the correct answer. The shaded quarter moves clockwise around the circle in each successive quadrant.</t>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Option B is the correct answer. The shaded quarter moves clockwise around the circle in each successive quadrant.</t>
   </si>
   <si>
     <t xml:space="preserve">Step 1: In the top-left quadrant, the top-left sector is shaded.
 Step 2: Moving clockwise to top-right, the shaded sector rotates 90 degrees clockwise.
 Step 3: In the bottom-left quadrant, the bottom-left sector is shaded.
-Step 4: Therefore, the missing 4th quadrant (bottom-right) must have the bottom-right sector shaded, which matches Option A.</t>
+Step 4: Therefore, the missing 4th quadrant (bottom-right) must have the bottom-right sector shaded, which matches Option B.</t>
   </si>
   <si>
     <t>Figure Series &amp; Rotations</t>
@@ -91,25 +91,28 @@
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20400%20100%22%20width%3D%22400%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22400%22%20height%3D%22100%22%20fill%3D%22%23f8fafc%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%2210%22%2F%3E%20%3C!--%20Box%201%3A%20UP%20(0%20deg)%20--%3E%20%3Crect%20x%3D%2210%22%20y%3D%2210%22%20width%3D%2280%22%20height%3D%2280%22%20fill%3D%22white%22%20stroke%3D%22%2394a3b8%22%20stroke-width%3D%222%22%20rx%3D%226%22%2F%3E%20%3Cline%20x1%3D%2250%22%20y1%3D%2270%22%20x2%3D%2250%22%20y2%3D%2225%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C15%2040%2C32%2060%2C32%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2272%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C!--%20Box%202%3A%20RIGHT%20(90%20deg)%20--%3E%20%3Crect%20x%3D%22105%22%20y%3D%2210%22%20width%3D%2280%22%20height%3D%2280%22%20fill%3D%22white%22%20stroke%3D%22%2394a3b8%22%20stroke-width%3D%222%22%20rx%3D%226%22%2F%3E%20%3Cline%20x1%3D%2225%22%20y1%3D%2250%22%20x2%3D%2270%22%20y2%3D%2250%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2285%2C50%2068%2C40%2068%2C60%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2223%22%20cy%3D%2250%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C!--%20Box%203%3A%20DOWN%20(180%20deg)%20--%3E%20%3Crect%20x%3D%22200%22%20y%3D%2210%22%20width%3D%2280%22%20height%3D%2280%22%20fill%3D%22white%22%20stroke%3D%22%2394a3b8%22%20stroke-width%3D%222%22%20rx%3D%226%22%2F%3E%20%3Cline%20x1%3D%22240%22%20y1%3D%2225%22%20x2%3D%22240%22%20y2%3D%2270%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%22240%2C85%20230%2C68%20250%2C68%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%22240%22%20cy%3D%2223%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C!--%20Box%204%3A%20%3F%20--%3E%20%3Crect%20x%3D%22295%22%20y%3D%2210%22%20width%3D%2295%22%20height%3D%2280%22%20fill%3D%22%23fef3c7%22%20stroke%3D%22%23f59e0b%22%20stroke-width%3D%222.5%22%20rx%3D%226%22%2F%3E%20%3Ctext%20x%3D%22342%22%20y%3D%2262%22%20font-size%3D%2244%22%20font-weight%3D%22900%22%20fill%3D%22%23dc2626%22%20text-anchor%3D%22middle%22%20font-family%3D%22sans-serif%22%3E%3F%3C%2Ftext%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cline%20x1%3D%2225%22%20y1%3D%2250%22%20x2%3D%2270%22%20y2%3D%2250%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2285%2C50%2068%2C40%2068%2C60%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2285%22%20cy%3D%2250%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cline%20x1%3D%2250%22%20y1%3D%2270%22%20x2%3D%2250%22%20y2%3D%2225%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C15%2040%2C32%2060%2C32%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2272%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cline%20x1%3D%2275%22%20y1%3D%2250%22%20x2%3D%2230%22%20y2%3D%2250%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2215%2C50%2032%2C40%2032%2C60%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2277%22%20cy%3D%2250%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cline%20x1%3D%2250%22%20y1%3D%2270%22%20x2%3D%2250%22%20y2%3D%2225%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C15%2040%2C32%2060%2C32%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2272%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cline%20x1%3D%2225%22%20y1%3D%2250%22%20x2%3D%2270%22%20y2%3D%2250%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2285%2C50%2068%2C40%2068%2C60%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2285%22%20cy%3D%2250%22%20r%3D%226%22%20fill%3D%22%2310b981%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cline%20x1%3D%2275%22%20y1%3D%2250%22%20x2%3D%2230%22%20y2%3D%2250%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2215%2C50%2032%2C40%2032%2C60%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>Option A is correct. The arrow rotates 90° clockwise in each step while keeping the green circle at its tail.</t>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Option C is correct. The arrow rotates 90° clockwise in each step while keeping the green circle at its tail.</t>
   </si>
   <si>
     <t xml:space="preserve">Step 1: Figure 1 points UP (0°).
 Step 2: Figure 2 points RIGHT (90° clockwise).
 Step 3: Figure 3 points DOWN (180° clockwise).
-Step 4: The 4th figure must point LEFT (270° clockwise) with the green marker at its tail, which is Option A.</t>
+Step 4: The 4th figure must point LEFT (270° clockwise) with the green marker at its tail, which is Option C.</t>
   </si>
   <si>
     <t>Mirror &amp; Water Images</t>
@@ -121,25 +124,25 @@
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20250%20120%22%20width%3D%22250%22%20height%3D%22120%22%3E%20%3Crect%20width%3D%22250%22%20height%3D%22120%22%20fill%3D%22%23f8fafc%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%2210%22%2F%3E%20%3C!--%20Question%20Figure%20on%20Left%20--%3E%20%3Crect%20x%3D%2230%22%20y%3D%2225%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%20rx%3D%226%22%2F%3E%20%3Cpath%20d%3D%22M%2045%2040%20L%2080%2040%20M%2045%2040%20L%2045%2080%20M%2045%2060%20L%2070%2060%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2285%2C40%2073%2C34%2073%2C46%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2245%22%20cy%3D%2280%22%20r%3D%225%22%20fill%3D%22%23f59e0b%22%2F%3E%20%3C!--%20Mirror%20Line%20MN%20--%3E%20%3Cline%20x1%3D%22160%22%20y1%3D%2210%22%20x2%3D%22160%22%20y2%3D%22110%22%20stroke%3D%22%23ef4444%22%20stroke-width%3D%223%22%20stroke-dasharray%3D%226%2C4%22%2F%3E%20%3Ctext%20x%3D%22160%22%20y%3D%2220%22%20font-size%3D%2212%22%20font-weight%3D%22900%22%20fill%3D%22%23ef4444%22%20text-anchor%3D%22middle%22%20dx%3D%2214%22%3EM%3C%2Ftext%3E%20%3Ctext%20x%3D%22160%22%20y%3D%22105%22%20font-size%3D%2212%22%20font-weight%3D%22900%22%20fill%3D%22%23ef4444%22%20text-anchor%3D%22middle%22%20dx%3D%2214%22%3EN%3C%2Ftext%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%20rx%3D%226%22%2F%3E%20%3Cpath%20d%3D%22M%2030%2030%20L%2065%2030%20M%2030%2030%20L%2030%2070%20M%2030%2050%20L%2055%2050%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2270%2C30%2058%2C24%2058%2C36%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2230%22%20cy%3D%2270%22%20r%3D%225%22%20fill%3D%22%23f59e0b%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%20rx%3D%226%22%2F%3E%20%3Cpath%20d%3D%22M%2055%2030%20L%2020%2030%20M%2055%2030%20L%2055%2070%20M%2055%2050%20L%2030%2050%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2215%2C30%2027%2C24%2027%2C36%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2255%22%20cy%3D%2270%22%20r%3D%225%22%20fill%3D%22%23f59e0b%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%20rx%3D%226%22%2F%3E%20%3Cpath%20d%3D%22M%2030%2030%20L%2065%2030%20M%2030%2030%20L%2030%2070%20M%2030%2050%20L%2055%2050%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2270%2C30%2058%2C24%2058%2C36%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2230%22%20cy%3D%2270%22%20r%3D%225%22%20fill%3D%22%23f59e0b%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%20rx%3D%226%22%2F%3E%20%3Cpath%20d%3D%22M%2055%2070%20L%2020%2070%20M%2055%2070%20L%2055%2030%20M%2055%2050%20L%2030%2050%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2215%2C70%2027%2C64%2027%2C76%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2255%22%20cy%3D%2230%22%20r%3D%225%22%20fill%3D%22%23f59e0b%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222.5%22%20rx%3D%226%22%2F%3E%20%3Cpath%20d%3D%22M%2030%2070%20L%2065%2070%20M%2030%2070%20L%2030%2030%20M%2030%2050%20L%2055%2050%22%20stroke%3D%22%232563eb%22%20stroke-width%3D%225%22%20stroke-linecap%3D%22round%22%2F%3E%20%3Cpolygon%20points%3D%2270%2C70%2058%2C64%2058%2C76%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2230%22%20cy%3D%2230%22%20r%3D%225%22%20fill%3D%22%23f59e0b%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>Option A is the correct mirror reflection. The arrow pointing right reflects to point left, while vertical positions remain unchanged.</t>
+    <t>Option B is the correct mirror reflection. The arrow pointing right reflects to point left, while vertical positions remain unchanged.</t>
   </si>
   <si>
     <t xml:space="preserve">Step 1: In lateral inversion across vertical mirror line MN, the left side becomes right and right becomes left.
 Step 2: The arrow pointing towards the right in the original figure points towards the left in the mirror image.
 Step 3: The yellow circle at bottom-left moves to bottom-right.
-Step 4: This matches Option A.</t>
+Step 4: This matches Option B.</t>
   </si>
   <si>
     <t>Embedded &amp; Hidden Figures</t>
@@ -161,6 +164,9 @@
   </si>
   <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C15%2085%2C85%2015%2C85%22%20fill%3D%22none%22%20stroke%3D%22%2394a3b8%22%20stroke-width%3D%222%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C40%2070%2C85%2030%2C85%22%20fill%3D%22none%22%20stroke%3D%22%2394a3b8%22%20stroke-width%3D%222%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
   <si>
     <t>Option A contains the exact Z-shaped profile embedded directly inside its grid lines.</t>
@@ -180,25 +186,28 @@
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20320%20100%22%20width%3D%22320%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22320%22%20height%3D%22100%22%20fill%3D%22%23f8fafc%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%2210%22%2F%3E%20%3C!--%20Step%201%3A%20Full%20Sheet%20--%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cline%20x1%3D%2250%22%20y1%3D%2215%22%20x2%3D%2250%22%20y2%3D%2285%22%20stroke%3D%22%23ef4444%22%20stroke-dasharray%3D%223%2C3%22%20stroke-width%3D%222%22%2F%3E%20%3C!--%20Arrow%201%20--%3E%20%3Cpath%20d%3D%22M%2092%2050%20L%20108%2050%22%20stroke%3D%22%2364748b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpolygon%20points%3D%22112%2C50%20104%2C46%20104%2C54%22%20fill%3D%22%2364748b%22%2F%3E%20%3C!--%20Step%202%3A%20Half%20Folded%20--%3E%20%3Crect%20x%3D%22120%22%20y%3D%2215%22%20width%3D%2235%22%20height%3D%2270%22%20fill%3D%22%23e2e8f0%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cline%20x1%3D%22120%22%20y1%3D%2250%22%20x2%3D%22155%22%20y2%3D%2250%22%20stroke%3D%22%23ef4444%22%20stroke-dasharray%3D%223%2C3%22%20stroke-width%3D%222%22%2F%3E%20%3C!--%20Arrow%202%20--%3E%20%3Cpath%20d%3D%22M%20165%2050%20L%20180%2050%22%20stroke%3D%22%2364748b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpolygon%20points%3D%22184%2C50%20176%2C46%20176%2C54%22%20fill%3D%22%2364748b%22%2F%3E%20%3C!--%20Step%203%3A%20Quarter%20with%20Hole%20Punched%20--%3E%20%3Crect%20x%3D%22195%22%20y%3D%2250%22%20width%3D%2235%22%20height%3D%2235%22%20fill%3D%22%23cbd5e1%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%22212%22%20cy%3D%2267%22%20r%3D%226%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C!--%20Arrow%203%20--%3E%20%3Cpath%20d%3D%22M%20240%2050%20L%20255%2050%22%20stroke%3D%22%2364748b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpolygon%20points%3D%22260%2C50%20252%2C46%20252%2C54%22%20fill%3D%22%2364748b%22%2F%3E%20%3C!--%20Step%204%3A%20Unfold%20%3F%20--%3E%20%3Crect%20x%3D%22270%22%20y%3D%2215%22%20width%3D%2238%22%20height%3D%2270%22%20fill%3D%22%23fef3c7%22%20stroke%3D%22%23f59e0b%22%20stroke-width%3D%222%22%20rx%3D%224%22%2F%3E%20%3Ctext%20x%3D%22289%22%20y%3D%2258%22%20font-size%3D%2228%22%20font-weight%3D%22900%22%20fill%3D%22%23dc2626%22%20text-anchor%3D%22middle%22%3E%3F%3C%2Ftext%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%227%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2265%22%20cy%3D%2265%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2235%22%20cy%3D%2250%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3Ccircle%20cx%3D%2265%22%20cy%3D%2250%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2235%22%20cy%3D%2235%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3Ccircle%20cx%3D%2265%22%20cy%3D%2235%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3Ccircle%20cx%3D%2235%22%20cy%3D%2265%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3Ccircle%20cx%3D%2265%22%20cy%3D%2265%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2265%22%20cy%3D%2265%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2235%22%20cy%3D%2250%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3Ccircle%20cx%3D%2265%22%20cy%3D%2250%22%20r%3D%225%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%227%22%20fill%3D%22%23dc2626%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
-    <t>Option A is correct. Unfolding the quarter sheet across both horizontal and vertical folds creates 4 symmetrical holes.</t>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Option D is correct. Unfolding the quarter sheet across both horizontal and vertical folds creates 4 symmetrical holes.</t>
   </si>
   <si>
     <t xml:space="preserve">Step 1: The paper is folded in half vertically, then in half horizontally (quarter sheet).
 Step 2: One circular hole is punched in this quarter.
 Step 3: Unfolding the first horizontal fold produces 2 holes.
-Step 4: Unfolding the vertical fold duplicates both holes to the other half, creating 4 symmetrical holes (Option A).</t>
+Step 4: Unfolding the vertical fold duplicates both holes to the other half, creating 4 symmetrical holes (Option D).</t>
   </si>
   <si>
     <t>Figure Analogy</t>
@@ -210,25 +219,25 @@
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20350%20100%22%20width%3D%22350%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22350%22%20height%3D%22100%22%20fill%3D%22%23f8fafc%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%2210%22%2F%3E%20%3C!--%20Pair%201%3A%20Figure%201%20-%3E%20Figure%202%20--%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2214%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ctext%20x%3D%2296%22%20y%3D%2258%22%20font-size%3D%2224%22%20font-weight%3D%22900%22%20fill%3D%22%2364748b%22%3E%3A%3C%2Ftext%3E%20%3Ccircle%20cx%3D%22145%22%20cy%3D%2250%22%20r%3D%2235%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Crect%20x%3D%22131%22%20y%3D%2236%22%20width%3D%2228%22%20height%3D%2228%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ctext%20x%3D%22195%22%20y%3D%2258%22%20font-size%3D%2224%22%20font-weight%3D%22900%22%20fill%3D%22%23dc2626%22%3E%3A%3A%3C%2Ftext%3E%20%3C!--%20Pair%202%3A%20Figure%203%20-%3E%20%3F%20--%3E%20%3Cpolygon%20points%3D%22255%2C15%20290%2C85%20220%2C85%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Ccircle%20cx%3D%22255%22%20cy%3D%2262%22%20r%3D%2212%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ctext%20x%3D%22298%22%20y%3D%2258%22%20font-size%3D%2224%22%20font-weight%3D%22900%22%20fill%3D%22%2364748b%22%3E%3A%3C%2Ftext%3E%20%3Crect%20x%3D%22310%22%20y%3D%2220%22%20width%3D%2230%22%20height%3D%2260%22%20fill%3D%22%23fef3c7%22%20stroke%3D%22%23f59e0b%22%20stroke-width%3D%222%22%20rx%3D%224%22%2F%3E%20%3Ctext%20x%3D%22325%22%20y%3D%2258%22%20font-size%3D%2224%22%20font-weight%3D%22900%22%20fill%3D%22%23dc2626%22%20text-anchor%3D%22middle%22%3E%3F%3C%2Ftext%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2235%22%20fill%3D%22%232563eb%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C30%2068%2C70%2032%2C70%22%20fill%3D%22white%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
+    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C30%2068%2C70%2032%2C70%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
+  </si>
+  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2235%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C30%2068%2C70%2032%2C70%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Crect%20x%3D%2215%22%20y%3D%2215%22%20width%3D%2270%22%20height%3D%2270%22%20fill%3D%22white%22%20stroke%3D%22%231e293b%22%20stroke-width%3D%222%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C30%2068%2C70%2032%2C70%22%20fill%3D%22%232563eb%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
-    <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2250%22%20r%3D%2235%22%20fill%3D%22%232563eb%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C30%2068%2C70%2032%2C70%22%20fill%3D%22white%22%2F%3E%20%3C%2Fsvg%3E</t>
-  </si>
-  <si>
     <t>data:image/svg+xml;utf8,%3Csvg%20xmlns%3D%22http%3A%2F%2Fwww.w3.org%2F2000%2Fsvg%22%20viewBox%3D%220%200%20100%20100%22%20width%3D%22100%22%20height%3D%22100%22%3E%20%3Crect%20width%3D%22100%22%20height%3D%22100%22%20fill%3D%22%23ffffff%22%20stroke%3D%22%23cbd5e1%22%20stroke-width%3D%222%22%20rx%3D%228%22%2F%3E%20%3Cpolygon%20points%3D%2250%2C15%2085%2C85%2015%2C85%22%20fill%3D%22%232563eb%22%2F%3E%20%3Ccircle%20cx%3D%2250%22%20cy%3D%2262%22%20r%3D%2212%22%20fill%3D%22white%22%2F%3E%20%3C%2Fsvg%3E</t>
   </si>
   <si>
-    <t>Option A is correct. The outer container and inner shape swap roles, with the new inner shape becoming solid blue.</t>
+    <t>Option C is correct. The outer container and inner shape swap roles, with the new inner shape becoming solid blue.</t>
   </si>
   <si>
     <t xml:space="preserve">Step 1: Figure 1 has a square outer boundary and a solid blue circle inside.
 Step 2: Figure 2 has a circle outer boundary and a solid blue square inside (roles swapped).
 Step 3: Figure 3 has a triangle outer boundary and a solid blue circle inside.
-Step 4: Therefore, the missing figure must have a circle outer boundary and a solid blue triangle inside (Option A).</t>
+Step 4: Therefore, the missing figure must have a circle outer boundary and a solid blue triangle inside (Option C).</t>
   </si>
 </sst>
 </file>
@@ -743,13 +752,13 @@
         <v>28</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -757,34 +766,34 @@
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>19</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" ht="70" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -792,34 +801,34 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -827,34 +836,34 @@
         <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -862,34 +871,34 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>